<commit_message>
(v3.0.1.9028) fix unique CIDs
</commit_message>
<xml_diff>
--- a/data-raw/datasets/antimicrobials.xlsx
+++ b/data-raw/datasets/antimicrobials.xlsx
@@ -9222,8 +9222,8 @@
           <t>CIX</t>
         </is>
       </c>
-      <c r="B145">
-        <v>47472</v>
+      <c r="B145" t="e">
+        <v>#N/A</v>
       </c>
       <c r="C145" t="inlineStr">
         <is>
@@ -18560,8 +18560,8 @@
           <t>NEO</t>
         </is>
       </c>
-      <c r="B296">
-        <v>8378</v>
+      <c r="B296" t="e">
+        <v>#N/A</v>
       </c>
       <c r="C296" t="inlineStr">
         <is>
@@ -20530,8 +20530,8 @@
           <t>PAS</t>
         </is>
       </c>
-      <c r="B328">
-        <v>4649</v>
+      <c r="B328" t="e">
+        <v>#N/A</v>
       </c>
       <c r="C328" t="inlineStr">
         <is>
@@ -26590,8 +26590,8 @@
           <t>SUM</t>
         </is>
       </c>
-      <c r="B426">
-        <v>5327</v>
+      <c r="B426" t="e">
+        <v>#N/A</v>
       </c>
       <c r="C426" t="inlineStr">
         <is>
@@ -27594,8 +27594,8 @@
           <t>SOX</t>
         </is>
       </c>
-      <c r="B442">
-        <v>5344</v>
+      <c r="B442" t="e">
+        <v>#N/A</v>
       </c>
       <c r="C442" t="inlineStr">
         <is>
@@ -29184,8 +29184,8 @@
           <t>TAT</t>
         </is>
       </c>
-      <c r="B468">
-        <v>9568512</v>
+      <c r="B468" t="e">
+        <v>#N/A</v>
       </c>
       <c r="C468" t="inlineStr">
         <is>
@@ -31064,8 +31064,8 @@
           <t>VIR</t>
         </is>
       </c>
-      <c r="B499">
-        <v>11979535</v>
+      <c r="B499" t="e">
+        <v>#N/A</v>
       </c>
       <c r="C499" t="inlineStr">
         <is>

</xml_diff>